<commit_message>
Let CO2 vary over the default 0.001-10 mM range instead of fixing it
Fixing CO2 at 10 mM made the malate shunt feasible but charged ~25 kJ/mol to
every CO2-producing step, costing the NfnAB pathway 1.8 kJ/mol. Leaving CO2
free over the default range gets both: the optimizer settles it low (~0.002-0.5
mM) in pathways that produce CO2 at PFOR, PDC or PDH, and high (~0.6-1.4 mM) in
the malate-shunt pathways that consume it at PEP carboxykinase.

All fifteen pathways remain feasible -- malate shunt modes at 2.78 and 4.40
kJ/mol -- and the PFOR-limited pathways return to their earlier values
(mode 4 at 6.57, mode 5 at 0.77). PFOR keeps 7.9 kJ/mol of surplus in the
native pathway, so the trapped-driving-force section is restored.

Caveat now stated in the README: CO2 is exchanged with the gas phase, so a real
fermentation would impose one shared value; letting it float per pathway is the
more permissive assumption.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ethanol_pathway_model.xlsx
+++ b/data/ethanol_pathway_model.xlsx
@@ -4482,14 +4482,14 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>10</v>
+        <v>0.001</v>
       </c>
       <c r="E31" t="n">
         <v>10</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Set to 10 mM, approximating dissolved CO2 in equilibrium with the fermentation gas phase. Dash et al. 2019 used a much lower value, which makes the malate shunt appear infeasible; Olson et al. 2017 showed that a ppdk deletion strain of C. thermocellum still produces ethanol, which requires the malate shunt, so the shunt must in fact be feasible.</t>
+          <t>Free over the default 0.001-10 mM range rather than fixed. Dash et al. 2019 used a low fixed value, at which the malate shunt is infeasible; Olson et al. 2017 showed a ppdk deletion strain still produces ethanol, which requires the malate shunt, so it must be feasible. Leaving CO2 free lets each pathway sit where its own thermodynamics allow. Note that CO2 is exchanged with the gas phase, so in a real fermentation all pathways would share one value.</t>
         </is>
       </c>
     </row>

</xml_diff>